<commit_message>
docs(order-management): confirm 24.5 scope — 7 routes, signed agreement, per-invoice PPL mirror; defer Booth Build; flag 24.5-h clause for BA
</commit_message>
<xml_diff>
--- a/order_management/24.5-quick-actions-per-order-item/24.5 - Quick Actions Per Order Item.xlsx
+++ b/order_management/24.5-quick-actions-per-order-item/24.5 - Quick Actions Per Order Item.xlsx
@@ -574,7 +574,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>11 requirement(s) to implement here (filter Build Focus = 'Implement here'). 0 covered elsewhere, 2 out of scope.</t>
+          <t>Scope confirmed 2026-07-03 — 10 requirement(s) to implement here (a,e,f,g,h,i,j,k,l,m). 24.5-d DEFERRED to the future Booth Build story (mirrors SBE-748); b/c out of scope; 24.5-h exhibitor-permissions clause flagged for BA removal. Jira: SBE-1129 (In Progress, Prantik Saha); branch feature/SBE-1129.</t>
         </is>
       </c>
     </row>
@@ -584,8 +584,10 @@
           <t>To implement here</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
-        <v>11</v>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
       </c>
     </row>
     <row r="6" ht="80" customHeight="1">
@@ -596,7 +598,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>This story asks for a per-order Quick Actions menu in Admin Panel &gt; Order Management exposing: open Upsell / Onsite Sale / Booth Build workflows (Booth Build gated to confirmed/signed orders + a Booth Build role); Download Agreement (Word + PDF); Download Order Invoice (PDF); Update Additional Users (admin adds emails, exhibitor sets permissions); Resend Order Confirm + Invoice; Resend Portal Password; and permission-based Log in to Customer Portal impersonation - with backend enforcement and logging. There is NO order/order-management module in any repo, so the whole admin endpoint surface is net-new, but re-verification against the actual code shows the underlying primitives are far more complete than previously assessed and most already live IN admin-backend-api: agreement download in BOTH PDF (buildSimplePdf) and Word (.doc) is fully built in the admin cart module; a generic mailer.sendFromTemplate plus seeded order-confirmation/welcome templates back the resend actions; admin impersonation already keys off company_id (finds the company's primary exhibitor, mints exhibitor JWTs, writes impersonated_by); the role/permission framework and audit/login logging are proven. Building the net-new order endpoints on these built primitives is therefore Deliverable for 10 of 13 requirements. Only Update Additional Users stays Partial (admin-add-emails is feasible via the invite primitive, but the 'permissions set by exhibitor' piece has no built company-user permission model). Upsell and Onsite Sale workflows belong to other epics and are Out of Scope as link targets.</t>
+          <t>This story asks for a per-order Quick Actions menu in Admin Panel &gt; Order Management exposing: open Upsell / Onsite Sale / Booth Build workflows (Booth Build gated to confirmed/signed orders + a Booth Build role); Download Agreement (Word + PDF); Download Order Invoice (PDF); Update Additional Users (admin adds emails, exhibitor sets permissions); Resend Order Confirm + Invoice; Resend Portal Password; and permission-based Log in to Customer Portal impersonation - with backend enforcement and logging. There is NO order/order-management module in any repo, so the whole admin endpoint surface is net-new, but re-verification against the actual code shows the underlying primitives are far more complete than previously assessed and most already live IN admin-backend-api: agreement download in BOTH PDF (buildSimplePdf) and Word (.doc) is fully built in the admin cart module; a generic mailer.sendFromTemplate plus seeded order-confirmation/welcome templates back the resend actions; admin impersonation already keys off company_id (finds the company's primary exhibitor, mints exhibitor JWTs, writes impersonated_by); the role/permission framework and audit/login logging are proven. Building the net-new order endpoints on these built primitives is therefore Deliverable for 10 of 13 requirements. Only Update Additional Users stays Partial (admin-add-emails is feasible via the invite primitive, but the 'permissions set by exhibitor' piece has no built company-user permission model). Upsell and Onsite Sale workflows belong to other epics and are Out of Scope as link targets. || SUPERSEDED AT SCOPE CONFIRMATION 2026-07-03: no /actions endpoint (per-route @Permissions is the enforcement); agreement download = the SIGNED contract (port exhibitor buildSignedBoothContractDocx; signed PDF net-new via pdfmake); invoice = per-invoice booth-layout renderer mirroring the admin PPL port (cache-first invoice_pdf_url); invite-user / impersonate port the shipped SBE-748 cart services; resend actions port the admin PPL pair (latest invoice PDF attached, throttled). 24.5-h flipped Partial → Deliverable; 24.5-d deferred.</t>
         </is>
       </c>
     </row>
@@ -630,8 +632,10 @@
           <t>Partial</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
-        <v>1</v>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -640,8 +644,10 @@
           <t>Blocked</t>
         </is>
       </c>
-      <c r="B11" s="6" t="n">
-        <v>0</v>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -672,7 +678,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Not started — analysis only</t>
+          <t>Not started — scope confirmed 2026-07-03; implementation plan next</t>
         </is>
       </c>
     </row>
@@ -830,12 +836,12 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>No order/order-management module or controller exists in any repo, so the admin endpoint that lists per-order actions is net-new - but the Order model and every primitive it needs (status, agreement, company, billing, cart link) exist and are populated. Building the net-new actions endpoint on these built primitives is Deliverable.</t>
+          <t>SCOPE DECISION 2026-07-03: no dedicated /actions endpoint. The menu is front-end; the backend contribution is the per-action routes on the shipped orders module (24.1–24.4), each gated by its own @Permissions key. Delivered by the union of 24.5-e/f/g/h/i/j/k routes + 24.5-l keys.</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/prisma/schema.prisma:1540 (model Order, incl. company_id, status, cart_id); codebase_map KEY STRUCTURAL FACTS (no order module exists)</t>
+          <t>shipped orders module src/admin/orders/orders.controller.ts (SBE-1125); guard pattern src/auth/guards/roles.guard.ts</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -852,7 +858,7 @@
       </c>
       <c r="L2" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started (no /actions endpoint — per-route guards)</t>
         </is>
       </c>
     </row>
@@ -990,7 +996,7 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Implement here</t>
+          <t>Deferred — future Booth Build story (2026-07-03)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -1026,7 +1032,7 @@
       </c>
       <c r="L5" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>Deferred 2026-07-03 — no gating code or permission key in this build; confirmed/signed mapping travels with the Booth Build story</t>
         </is>
       </c>
     </row>
@@ -1058,12 +1064,12 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>PRIOR GAP DISPROVEN: a working Word (.doc) agreement generator already exists IN admin-backend-api - AgreementDocumentService.generate(id,'docx') emits application/msword HTML from live cart line items, pricing, fees and additional_terms, and is already wired to a download route. Orders are created from carts (Order.cart_id), so the net-new work is an order-scoped endpoint reusing this built generator.</t>
+          <t>SCOPE DECISION 2026-07-03: download the SIGNED contract, not the unsigned live-cart draft. Port exhibitor buildSignedBoothContractDocx (Order snapshot + frozen agreement_ids terms + FILLED signature block, S3 cache-first on OrderAgreement.signed_agreement_url) into the orders module — admin ppl-order already proved this port pattern.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/admin/cart/services/agreement-document.service.ts:29 (generate pdf|docx), :41-45 (.doc via buildWordHtml); admin/cart/cart.controller.ts:1141 (@Get :id/agreement.docx, @Permissions)</t>
+          <t>exhibitor agreement.service.ts:1429 (buildSignedBoothContractDocx); admin port precedent admin/ppl-order/services/agreement-document.service.ts:29; OrderAgreement.signed_agreement_url (shared cache)</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1084,7 +1090,7 @@
       </c>
       <c r="L6" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started (signed DOCX port)</t>
         </is>
       </c>
     </row>
@@ -1116,12 +1122,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>PRIOR GAP DISPROVEN: the prior analysis claimed 'no PDF agreement renderer exists anywhere' - it does. admin-backend-api renders the agreement PDF via the dependency-free buildSimplePdf util, exposed today at the cart agreement.pdf route. Same content as the Word export. Net-new work is the order-scoped endpoint reusing the built PDF renderer.</t>
+          <t>SCOPE DECISION 2026-07-03: signed-contract PDF. No signed-PDF renderer exists anywhere (signed builders are DOCX-only; the cart PDF is the unsigned draft) — net-new pdfmake composition over the same order-snapshot context as 24.5-e, built here (Confluence requires both formats). signed_agreement_url caches DOCX only; PDF caching decided at plan time.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/admin/cart/utils/pdf.util.ts:49 (buildSimplePdf); agreement-document.service.ts:33-38 (pdf branch); admin/cart/cart.controller.ts:1122 (@Get :id/agreement.pdf)</t>
+          <t>admin PdfmakeService usage cart/services/agreement-document.service.ts:146-147; no signed-PDF renderer found in any repo</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
@@ -1142,7 +1148,7 @@
       </c>
       <c r="L7" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started (net-new signed PDF)</t>
         </is>
       </c>
     </row>
@@ -1174,12 +1180,12 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Invoice rows are actually written by the Stripe webhook for both PPL and booth orders (shared DB), a proven invoice-PDF renderer exists (exhibitor pdfkit renderInvoicePdf), and admin itself already renders PDFs (buildSimplePdf). The net-new work is an admin order endpoint that loads the order's Invoice rows and streams a PDF - Deliverable on built primitives.</t>
+          <t>SCOPE DECISION 2026-07-03: per-invoice route mirroring the shipped PPL shape (booth orders create one Invoice per successful installment). Admin's ported InvoiceDocumentService provides pdfkit + cache-first Invoice.invoice_pdf_url + getPdfBufferForAttachment; net-new = the booth/product layout branch over the typed line-item tree the webhook already snapshots.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Invoice written external-api-service/src/modules/webhook/services/webhook.service.ts:679,2048; renderer exhibitor-backend-api/src/ppl/services/ppl.service.ts:985 (renderInvoicePdf); admin PDF util pdf.util.ts:49; model Invoice schema.prisma:1962</t>
+          <t>admin/ppl-order/services/invoice-document.service.ts; route shape ppl-order.controller.ts:90; tree snapshot external-api webhook.service.ts:2054-2075</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -1196,7 +1202,7 @@
       </c>
       <c r="L8" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started (booth layout branch)</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1219,7 @@
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Deliverable</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1228,12 +1234,12 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>The admin-adds-emails half is feasible: the full invite primitive (create Exhibitor row + ExhibitorToken + send invitation email) is built and admin has the mailer to drive it (current invite is exhibitor primary-only, so an admin variant is net-new). The genuine gap is the 'permissions set by exhibitor' half - the company_user service exposes only invite/accept/resend/revoke/toggle-status; there is NO company-user permission/access-level model or endpoint for the exhibitor to set per-user permissions, so that capability is not built.</t>
+          <t>RE-VERDICTED 2026-07-03 (was Partial): admin already ships the complete invite flow as the SBE-748 cart quick action (CartInviteUserService behind POST /carts/:id/invite-user — portal user + token + company_user_invitation template + audit). Order variant delegates the same flow keyed off order.company_id. The former gap ('permissions set by exhibitor') is FLAGGED FOR BA REMOVAL — no company-user permission model exists anywhere; the cart-management section has no such clause either.</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>exhibitor-backend-api/src/company_user/company_user.controller.ts:49 (invite, primary-only), :254 (resend), :384 (list); company_user.service.ts:238 (exhibitor.create), :265 (exhibitorToken.create) - no permission-setting found in company_user.service.ts</t>
+          <t>admin/cart/services/cart-invite-user.service.ts; cart.controller.ts:1118 (@Post :id/invite-user)</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
@@ -1250,7 +1256,7 @@
       </c>
       <c r="L9" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started (port of cart invite; BA flag on exhibitor clause)</t>
         </is>
       </c>
     </row>
@@ -1282,12 +1288,12 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Admin has a generic template dispatcher (mailer.sendFromTemplate, already used by resendWelcome) and the order-confirmation templates (ppl_order_confirmation, booth_order_confirmation) are seeded in admin. A net-new admin resend endpoint that composes order data and calls sendFromTemplate is Deliverable on built primitives. (Today these templates merge the invoice number as text - whether a PDF must additionally be attached is the one open question.)</t>
+          <t>Former attach-PDF open question RESOLVED by in-repo precedent: admin PPL resendOrderConfirmation already attaches the latest invoice PDF (getPdfBufferForAttachment) behind a throttle window. Booth port resends the seeded booth_order_confirmation with the latest invoice PDF from 24.5-g's renderer.</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>admin mailer.sendFromTemplate admin-backend-api/src/admin/exhibitor-management/exhibitor-management.service.ts:448; templates admin-backend-api/src/database/seeds/notification-template.seeder.ts:93,142; existing send path external-api-service/src/modules/webhook/services/webhook.service.ts:1850,2531 (merges invoice_number)</t>
+          <t>admin/ppl-order/services/ppl-order-actions.service.ts:184-225 (resend + attach + throttle)</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
@@ -1308,7 +1314,7 @@
       </c>
       <c r="L10" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started (port of PPL resend)</t>
         </is>
       </c>
     </row>
@@ -1340,12 +1346,12 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>All primitives are built: admin already issues a fresh password + email via resendWelcome (mailer.sendFromTemplate + bcrypt + notificationLog dedupe), and the exhibitor portal has a full forgot/reset-password flow (token issue + reset email). A net-new admin order endpoint triggering a portal password reset/temp-password email is Deliverable on these built primitives.</t>
+          <t>CLOSEST PRECEDENT (2026-07-03): admin PPL already ships this exact action — resendPortalPassword sending the admin_resend_portal_access template. Order variant = port keyed on the order's company primary exhibitor.</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>admin resendWelcome exhibitor-backend-api... admin-backend-api/src/admin/exhibitor-management/exhibitor-management.service.ts:277 (resendWelcome), :448 (mailer.sendFromTemplate); exhibitor reset flow exhibitor-backend-api/src/auth/controllers/auth.controller.ts:294 (exhibitor-forgot-password)</t>
+          <t>admin/ppl-order/services/ppl-order-actions.service.ts:341, :49 (template)</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
@@ -1366,7 +1372,7 @@
       </c>
       <c r="L11" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started (port of PPL portal-password resend)</t>
         </is>
       </c>
     </row>
@@ -1398,12 +1404,12 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>PRIOR 'PPL-only' CAVEAT CORRECTED: the impersonation primitive already keys off company_id - it finds the company's primary exhibitor (user_type=1), mints SBEEXHIBITOR access/refresh JWTs, is @Permissions-gated, and writes impersonated_by to the login log. An Order carries company_id, so the net-new admin order endpoint reuses this generic, built primitive directly.</t>
+          <t>CLOSEST PRECEDENT (2026-07-03): the SBE-748 cart quick action already ships this — CartImpersonateService behind POST /carts/:id/impersonate (company → primary exhibitor → exhibitor JWTs → impersonated_by + activity log). Order variant = same pattern keyed off order.company_id.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>admin-backend-api/src/admin/ppl-service-provider-overview/ppl-service-provider-overview.service.ts:320 (impersonate({company_id})), :339-341 (find primary exhibitor by company_id), :400 (signAsync JWTs), :431 (impersonated_by login log); controller :153 (@Get impersonate, @Permissions)</t>
+          <t>admin/cart/services/cart-impersonate.service.ts:70,:187,:202; cart.controller.ts:1026</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -1420,7 +1426,7 @@
       </c>
       <c r="L12" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started (port of cart impersonate)</t>
         </is>
       </c>
     </row>
@@ -1478,7 +1484,7 @@
       </c>
       <c r="L13" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started (per-route permission keys + role grants + Swagger docs; no availability endpoint)</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1538,7 @@
       </c>
       <c r="L14" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started</t>
+          <t>◻ Not started (delivered by construction via ported services' logs; verified at smoke)</t>
         </is>
       </c>
     </row>
@@ -1563,7 +1569,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1608,20 +1614,24 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/orders/:id/actions</t>
+          <t>/api/v1/orders/:id/agreement.docx</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Return the permission- and status-gated set of quick actions for an order (Booth Build only when completed/signed and caller has the Booth Build role).</t>
+          <t>Stream the SIGNED booth contract DOCX (Order snapshot + frozen terms + filled signature block); cache-first on OrderAgreement.signed_agreement_url.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>24.5-a, 24.5-d, 24.5-l</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+          <t>24.5-e</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>24.6 — same endpoint serves 24.6-s. Cache shared with the exhibitor signed download.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1631,22 +1641,22 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/orders/:id/agreement.docx</t>
+          <t>/api/v1/orders/:id/agreement.pdf</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Stream the order agreement as Word (.docx) reflecting booth details/pricing/terms.</t>
+          <t>Stream the SIGNED contract as PDF (net-new pdfmake composition over the same order-snapshot context).</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>24.5-e</t>
+          <t>24.5-f</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>24.6 — same agreement endpoint serves 24.6-s (view/download agreement).</t>
+          <t>24.6 — same endpoint serves 24.6-s.</t>
         </is>
       </c>
     </row>
@@ -1658,44 +1668,40 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/orders/:id/agreement.pdf</t>
+          <t>/api/v1/orders/:id/invoices/:invoiceId/invoice</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Stream the order agreement as PDF.</t>
+          <t>Generate (or return cached) the invoice PDF for an invoice belonging to the order — booth/product layout over the typed line-item tree; mirrors the shipped PPL route.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>24.5-f</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>24.6 — same agreement endpoint serves 24.6-s (view/download agreement).</t>
-        </is>
-      </c>
+          <t>24.5-g</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/orders/:id/invoice.pdf</t>
+          <t>/api/v1/orders/:id/invite-user</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Stream the order invoice PDF from the order's written Invoice rows.</t>
+          <t>Admin adds a portal-user email ID for the order's company (invitation token + email; one email per call, mirrors the SBE-748 cart action).</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>24.5-g</t>
+          <t>24.5-h</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr"/>
@@ -1708,17 +1714,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/orders/:id/additional-users</t>
+          <t>/api/v1/orders/:id/resend-confirmation</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Admin adds one or more portal-user email IDs for the order's company (invitation sent; permissions set later by the exhibitor).</t>
+          <t>Resend booth_order_confirmation with the latest invoice PDF attached (throttled).</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>24.5-h</t>
+          <t>24.5-i</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -1731,17 +1737,17 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/orders/:id/resend-confirmation</t>
+          <t>/api/v1/orders/:id/resend-portal-password</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Resend the order confirmation email (with invoice details) to the customer.</t>
+          <t>Send the admin_resend_portal_access portal password email for the order's customer (logged).</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>24.5-i</t>
+          <t>24.5-j, 24.5-m</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -1754,43 +1760,20 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>/api/v1/orders/:id/resend-portal-password</t>
+          <t>/api/v1/orders/:id/impersonate</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Trigger a portal password-reset / temp-password email for the order's customer (logged).</t>
+          <t>Permission-based login as the order company's primary exhibitor (exhibitor JWTs), logged via impersonated_by.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>24.5-j, 24.5-m</t>
+          <t>24.5-k, 24.5-m</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>/api/v1/orders/:id/impersonate</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Permission-based login as the order company's primary exhibitor (mint exhibitor portal JWTs), logged via impersonated_by.</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>24.5-k, 24.5-m</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1803,7 +1786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1845,12 +1828,12 @@
       </c>
       <c r="C2" s="14" t="inlineStr">
         <is>
-          <t>[OPEN — for team discussion]</t>
+          <t>[CLOSED 2026-07-03 — moot by deferral]</t>
         </is>
       </c>
       <c r="D2" s="14" t="inlineStr">
         <is>
-          <t>Current direction (2026-07-01): lean toward mapping 'confirmed' -&gt; status = completed and 'signed' -&gt; presence of an OrderAgreement row (written at checkout sign); OrderStatus has no literal 'confirmed'. Pending team confirmation before 24.5-d gating code.</t>
+          <t>24.5-d deferred to the future Booth Build story (mirrors SBE-748); the confirmed/signed mapping question travels with that story and no longer gates anything here.</t>
         </is>
       </c>
     </row>
@@ -1865,12 +1848,34 @@
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>[OPEN — for team discussion]</t>
+          <t>[RESOLVED 2026-07-03 — in-repo precedent]</t>
         </is>
       </c>
       <c r="D3" s="14" t="inlineStr">
         <is>
-          <t>Current direction (2026-07-01): pending. Team to confirm whether the resend must attach the generated invoice PDF or whether the merged invoice-number text suffices. Scope of 24.5-i depends on the answer.</t>
+          <t>Attach the PDF: admin PPL resendOrderConfirmation already attaches the latest invoice PDF behind a throttle window; the booth port does the same using 24.5-g's renderer.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>24.5-h clause 'access permission shall be set by the exhibitor' — no company-user permission model exists in any repo, and the cart-management section (18.6/19.6, SBE-748) has no such concept.</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>[NEW — for BA]</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Flagged for BA removal from the story (2026-07-03); not counted as a build gap.</t>
         </is>
       </c>
     </row>
@@ -1999,7 +2004,7 @@
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>Not started — analysis/feasibility stage only. No branch, no SBE ticket, no PR, no Swagger tag. Entire admin order-actions surface is net-new (no order/order-management module exists in any repo).</t>
+          <t>Scope confirmed 2026-07-03 (Step 1 done; plan next). Jira SBE-1129 (In Progress, Prantik Saha); branch feature/SBE-1129 to cut. Nothing built yet — all 10 in-scope reqs ◻ Not started.</t>
         </is>
       </c>
     </row>
@@ -2011,7 +2016,7 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>— (not started).</t>
+          <t>feature/SBE-1129 (to cut from dev)</t>
         </is>
       </c>
     </row>
@@ -2023,31 +2028,31 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>All 11 in-scope reqs un-built: 24.5-a,d,e,f,g,h,i,j,k,l,m are ◻ Not started. 24.5-h stays Partial (admin-add-emails feasible; 'permissions set by exhibitor' half has no built model).</t>
+          <t>All 10 in-scope reqs un-built: 24.5-a,e,f,g,h,i,j,k,l,m. 24.5-d deferred (not remaining here); 24.5-h exhibitor clause = BA-removal flag, not remaining work.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>Open decision — Booth Build gating</t>
+          <t>Closed decision — Booth Build gating</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>Confirm 'confirmed' -&gt; status = completed and 'signed' -&gt; presence of an OrderAgreement row. Gates 24.5-d. No code until answered.</t>
+          <t>Moot 2026-07-03: 24.5-d deferred to the future Booth Build story; the mapping question travels with it.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Open decision — resend invoice PDF</t>
+          <t>Closed decision — resend invoice PDF</t>
         </is>
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>Confirm whether Resend Order Confirm and Invoice must attach the generated invoice PDF vs merging the invoice number as text. Affects 24.5-i. No code until answered.</t>
+          <t>Resolved 2026-07-03 by in-repo precedent: attach the latest invoice PDF (admin PPL resend already does; throttled).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(order-management): record 24.5 implementation — built on feature/SBE-1125 (3624d09), review register added, PR pending
</commit_message>
<xml_diff>
--- a/order_management/24.5-quick-actions-per-order-item/24.5 - Quick Actions Per Order Item.xlsx
+++ b/order_management/24.5-quick-actions-per-order-item/24.5 - Quick Actions Per Order Item.xlsx
@@ -678,7 +678,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Not started — scope confirmed 2026-07-03; implementation plan next</t>
+          <t>IMPLEMENTED 2026-07-03 — Phase 0 10/10, live smoke 15 checks, formal 8-angle code review (all 10 confirmed findings fixed + regression-tested), pre-push gate 8/8 (2877 tests, cov 94.95%/81.41%). PR not yet raised (user-driven).</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>feature/SBE-1125</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>admin 3624d09 feat(SBE-1129) — 15 files; ZERO schema changes, no sibling-repo syncs</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>not raised yet (user-driven); pipelines are PR-triggered</t>
         </is>
       </c>
     </row>
@@ -858,7 +858,7 @@
       </c>
       <c r="L2" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started (no /actions endpoint — per-route guards)</t>
+          <t>✅ Implemented — 7 per-route @Permissions endpoints ARE the backend (no /actions); live Swagger verified</t>
         </is>
       </c>
     </row>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="L5" s="14" t="inlineStr">
         <is>
-          <t>Deferred 2026-07-03 — no gating code or permission key in this build; confirmed/signed mapping travels with the Booth Build story</t>
+          <t>Deferred — future Booth Build story (no code, no key)</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1090,7 @@
       </c>
       <c r="L6" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started (signed DOCX port)</t>
+          <t>✅ Implemented — OrderAgreementDocumentService DOCX port, shared signed_agreement_url cache; render parity review-verified</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="L7" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started (net-new signed PDF)</t>
+          <t>✅ Implemented — net-new signed-PDF pdfmake composition (no cache, D3); terms heading fixed at review</t>
         </is>
       </c>
     </row>
@@ -1202,7 +1202,7 @@
       </c>
       <c r="L8" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started (booth layout branch)</t>
+          <t>✅ Implemented — per-invoice PPL mirror + booth tree layout; local smoke blocked at S3 upload boundary (env IAM — register)</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="L9" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started (port of cart invite; BA flag on exhibitor clause)</t>
+          <t>✅ Implemented — POST :id/invite-user cart port; smoke 201 + token + email; BA flag stands on exhibitor clause</t>
         </is>
       </c>
     </row>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="L10" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started (port of PPL resend)</t>
+          <t>✅ Implemented — booth_order_confirmation + latest invoice PDF attached; SENT-only throttle; smoke verified</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
       </c>
       <c r="L11" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started (port of PPL portal-password resend)</t>
+          <t>✅ Implemented — admin_resend_portal_access port; delivery now VERIFIED (502 on silent failure) per review fix</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="L12" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started (port of cart impersonate)</t>
+          <t>✅ Implemented — cart impersonate port; SBEEXHIBITOR_* cookies + impersonated_by session (psql-verified)</t>
         </is>
       </c>
     </row>
@@ -1484,7 +1484,7 @@
       </c>
       <c r="L13" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started (per-route permission keys + role grants + Swagger docs; no availability endpoint)</t>
+          <t>✅ Implemented — 6 orders.* keys seeded/granted/Swagger-documented; RawParam+ParseIntIdPipe on all ids (review fix)</t>
         </is>
       </c>
     </row>
@@ -1538,7 +1538,7 @@
       </c>
       <c r="L14" s="14" t="inlineStr">
         <is>
-          <t>◻ Not started (delivered by construction via ported services' logs; verified at smoke)</t>
+          <t>✅ Implemented — 6 order-entity audit rows (best-effort writes), impersonated_by, activity/notification logs</t>
         </is>
       </c>
     </row>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>Scope confirmed 2026-07-03 (Step 1 done; plan next). Jira SBE-1129 (In Progress, Prantik Saha); branch feature/SBE-1129 to cut. Nothing built yet — all 10 in-scope reqs ◻ Not started.</t>
+          <t>IMPLEMENTED 2026-07-03 on feature/SBE-1125, admin commit 3624d09 (15 files, zero schema changes). Phase 0 10/10; live smoke 15 checks (signed DOCX/PDF content-verified, invite/impersonate/resends with DB-level evidence, teardown done); formal code review: 8 finder angles, 24 verified candidates, all 10 confirmed findings FIXED + regression-tested; pre-push gate 8/8 (2877 tests, cov 94.95%/81.41%). PR not yet raised (user-driven).</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>feature/SBE-1129 (to cut from dev)</t>
+          <t>feature/SBE-1125 — admin 3624d09 feat(SBE-1129)</t>
         </is>
       </c>
     </row>
@@ -2028,7 +2028,7 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>All 10 in-scope reqs un-built: 24.5-a,e,f,g,h,i,j,k,l,m. 24.5-d deferred (not remaining here); 24.5-h exhibitor clause = BA-removal flag, not remaining work.</t>
+          <t>Lifecycle only: raise PR vs dev (user) → pipeline/Sonar loop → merge (delivers 24.6-s's backend). Review register in the .md: 4 fixed-here-but-live-in-shipped-twins items (cart/PPL sources need the same patches), 4 accepted below-cap items, 15 cleanup/tech-debt opportunities, 2 local-env gaps (S3 PutObject IAM; EXHIBITOR_JWT secrets).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(order-management): 24.5 PR#521 green — dev-unblock fix, toolchain hoist, pipeline #856 + Sonar OK
</commit_message>
<xml_diff>
--- a/order_management/24.5-quick-actions-per-order-item/24.5 - Quick Actions Per Order Item.xlsx
+++ b/order_management/24.5-quick-actions-per-order-item/24.5 - Quick Actions Per Order Item.xlsx
@@ -678,7 +678,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IMPLEMENTED 2026-07-03 — Phase 0 10/10, live smoke 15 checks, formal 8-angle code review (all 10 confirmed findings fixed + regression-tested), pre-push gate 8/8 (2877 tests, cov 94.95%/81.41%). PR not yet raised (user-driven).</t>
+          <t>IMPLEMENTED 2026-07-03 — Phase 0 10/10, live smoke 15 checks, formal review (10 findings fixed), pre-push gate 8/8; PR#521 pipeline #856 SUCCESSFUL + SonarQube gate OK (3001 tests, cov 95.02%/81.19%). Merge pending.</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>admin 3624d09 feat(SBE-1129) — 15 files; ZERO schema changes, no sibling-repo syncs</t>
+          <t>admin e06e860 feat + 161aae8 test (dev-unblocking id-walker guard fix, our own) + adeba9f refactor (shared BaseAgreementDocumentService hoist; cart service now extends it too). ZERO schema changes.</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>not raised yet (user-driven); pipelines are PR-triggered</t>
+          <t>PR#521 raised 2026-07-03 — pipeline #856 SUCCESSFUL, Sonar gate OK. Merge pending team.</t>
         </is>
       </c>
     </row>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>IMPLEMENTED 2026-07-03 on feature/SBE-1125, admin commit 3624d09 (15 files, zero schema changes). Phase 0 10/10; live smoke 15 checks (signed DOCX/PDF content-verified, invite/impersonate/resends with DB-level evidence, teardown done); formal code review: 8 finder angles, 24 verified candidates, all 10 confirmed findings FIXED + regression-tested; pre-push gate 8/8 (2877 tests, cov 94.95%/81.41%). PR not yet raised (user-driven).</t>
+          <t>IMPLEMENTED 2026-07-03 on feature/SBE-1125, admin commit 3624d09 (15 files, zero schema changes). Phase 0 10/10; live smoke 15 checks (signed DOCX/PDF content-verified, invite/impersonate/resends with DB-level evidence, teardown done); formal code review: 8 finder angles, 24 verified candidates, all 10 confirmed findings FIXED + regression-tested; pre-push gate 8/8 (2877 tests, cov 94.95%/81.41%). PR#521 raised: first run #851 failed on PRE-EXISTING dev breakage (PR#455 guard x PR#518 cyclic DTO — we shipped our own fix 161aae8, unblocking all PRs); #855 failed Sonar (1 smell fixed + duplication gate -&gt; toolchain hoisted to shared base, adeba9f); #856 SUCCESSFUL + Sonar OK. Merge pending.</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>feature/SBE-1125 — admin 3624d09 feat(SBE-1129)</t>
+          <t>feature/SBE-1125 — admin e06e860 / 161aae8 / adeba9f (rebased onto dev)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(order-management): 24.5 merged to dev — story complete; 24.6-s delivered; C6 shipped w/ shared toolchain note
</commit_message>
<xml_diff>
--- a/order_management/24.5-quick-actions-per-order-item/24.5 - Quick Actions Per Order Item.xlsx
+++ b/order_management/24.5-quick-actions-per-order-item/24.5 - Quick Actions Per Order Item.xlsx
@@ -678,7 +678,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>IMPLEMENTED 2026-07-03 — Phase 0 10/10, live smoke 15 checks, formal review (10 findings fixed), pre-push gate 8/8; PR#521 pipeline #856 SUCCESSFUL + SonarQube gate OK (3001 tests, cov 95.02%/81.19%). Merge pending.</t>
+          <t>IMPLEMENTED 2026-07-03 — smoke 15, formal review (10 findings fixed), gate 8/8; PR#521 pipeline #856 + Sonar OK; MERGED to dev 2026-07-03 (34c6fb4). STORY COMPLETE.</t>
         </is>
       </c>
     </row>
@@ -714,7 +714,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>PR#521 raised 2026-07-03 — pipeline #856 SUCCESSFUL, Sonar gate OK. Merge pending team.</t>
+          <t>PR#521 MERGED to dev 2026-07-03 (34c6fb4); pipeline #856 SUCCESSFUL, Sonar gate OK.</t>
         </is>
       </c>
     </row>
@@ -2004,7 +2004,7 @@
       </c>
       <c r="B2" s="14" t="inlineStr">
         <is>
-          <t>IMPLEMENTED 2026-07-03 on feature/SBE-1125, admin commit 3624d09 (15 files, zero schema changes). Phase 0 10/10; live smoke 15 checks (signed DOCX/PDF content-verified, invite/impersonate/resends with DB-level evidence, teardown done); formal code review: 8 finder angles, 24 verified candidates, all 10 confirmed findings FIXED + regression-tested; pre-push gate 8/8 (2877 tests, cov 94.95%/81.41%). PR#521 raised: first run #851 failed on PRE-EXISTING dev breakage (PR#455 guard x PR#518 cyclic DTO — we shipped our own fix 161aae8, unblocking all PRs); #855 failed Sonar (1 smell fixed + duplication gate -&gt; toolchain hoisted to shared base, adeba9f); #856 SUCCESSFUL + Sonar OK. Merge pending.</t>
+          <t>IMPLEMENTED 2026-07-03 on feature/SBE-1125, admin commit 3624d09 (15 files, zero schema changes). Phase 0 10/10; live smoke 15 checks (signed DOCX/PDF content-verified, invite/impersonate/resends with DB-level evidence, teardown done); formal code review: 8 finder angles, 24 verified candidates, all 10 confirmed findings FIXED + regression-tested; pre-push gate 8/8 (2877 tests, cov 94.95%/81.41%). PR#521 raised: first run #851 failed on PRE-EXISTING dev breakage (PR#455 guard x PR#518 cyclic DTO — we shipped our own fix 161aae8, unblocking all PRs); #855 failed Sonar (1 smell fixed + duplication gate -&gt; toolchain hoisted to shared base, adeba9f); #856 SUCCESSFUL + Sonar OK; MERGED to dev 2026-07-03 (34c6fb4). STORY COMPLETE.</t>
         </is>
       </c>
     </row>
@@ -2028,7 +2028,7 @@
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>Lifecycle only: raise PR vs dev (user) → pipeline/Sonar loop → merge (delivers 24.6-s's backend). Review register in the .md: 4 fixed-here-but-live-in-shipped-twins items (cart/PPL sources need the same patches), 4 accepted below-cap items, 15 cleanup/tech-debt opportunities, 2 local-env gaps (S3 PutObject IAM; EXHIBITOR_JWT secrets).</t>
+          <t>None — merged. 24.6-s delivered on dev. Review register items for the team stand (see .md).</t>
         </is>
       </c>
     </row>

</xml_diff>